<commit_message>
privacidad: reglas 2, 3, 5 y 7 aprobadas, limpieza de datos de terceros y cron mensual
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clientes/tamarama/Mangueras_Xiandai_vs_Dongying.xlsx
+++ b/clientes/tamarama/Mangueras_Xiandai_vs_Dongying.xlsx
@@ -26,13 +26,13 @@
     <t>Proveedor nuevo</t>
   </si>
   <si>
-    <t>Weifang Xiandai Plastics &amp; Rubbers (Lina Liu) · cotización XDQ260916 del 16-sep-2026</t>
+    <t>Weifang Xiandai Plastics &amp; Rubbers · cotización XDQ260916 del 16-sep-2026</t>
   </si>
   <si>
     <t>Proveedor anterior</t>
   </si>
   <si>
-    <t>Dongying Wanhe Rubber &amp; Plastic (Ben Hu) · último precio: proforma DYWH20210607CH01 del 7-jun-2021</t>
+    <t>Dongying Wanhe Rubber &amp; Plastic · último precio: proforma DYWH20210607CH01 del 7-jun-2021</t>
   </si>
   <si>
     <t>Motivo del cambio</t>
@@ -242,7 +242,7 @@
     <t>Un contenedor 40HQ tiene unos 76 m³ interiores (~68 m³ útiles). Con Xiandai el mismo pedido no cabe: ajustar el mix o pedir su plan de carga.</t>
   </si>
   <si>
-    <t>Lo que falta pedirle a Lina (Xiandai)</t>
+    <t>Lo que falta pedirle a Xiandai</t>
   </si>
   <si>
     <t>Pedido por Pedro el 14-sep y no entregado, más lo recomendado</t>

</xml_diff>